<commit_message>
chore: sync from game project — WYSIWYG 命名重构、PascalCase 重命名、UIConfig/ja 导出、AGENTS.md 桥接
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gd/excel/item.xlsx
+++ b/gd/excel/item.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="item" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Item" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -70,7 +70,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -84,11 +84,53 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -103,6 +145,8 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -502,7 +546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -519,244 +563,74 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <rFont val="Segoe UI"/>
-              <b val="1"/>
-              <color rgb="00FFFFFF"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">id
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Consolas"/>
-              <i val="1"/>
-              <color rgb="00D8F3DC"/>
-              <sz val="9"/>
-            </rPr>
-            <t>int32</t>
-          </r>
+          <t>Id
+int32</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <rFont val="Segoe UI"/>
-              <b val="1"/>
-              <color rgb="00FFFFFF"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">name
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Consolas"/>
-              <i val="1"/>
-              <color rgb="00D8F3DC"/>
-              <sz val="9"/>
-            </rPr>
-            <t>string[i18n]</t>
-          </r>
+          <t>Name
+string[i18n]</t>
         </is>
       </c>
       <c r="C1" s="2" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <rFont val="Segoe UI"/>
-              <b val="1"/>
-              <color rgb="00FFFFFF"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">price
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Consolas"/>
-              <i val="1"/>
-              <color rgb="00D8F3DC"/>
-              <sz val="9"/>
-            </rPr>
-            <t>float</t>
-          </r>
+          <t>Price
+float</t>
         </is>
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <rFont val="Segoe UI"/>
-              <b val="1"/>
-              <color rgb="00FFFFFF"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">rarity
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Consolas"/>
-              <i val="1"/>
-              <color rgb="00D8F3DC"/>
-              <sz val="9"/>
-            </rPr>
-            <t>enum[common,rare,epic]</t>
-          </r>
+          <t>Rarity
+enum[common,rare,epic]</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <rFont val="Segoe UI"/>
-              <b val="1"/>
-              <color rgb="00FFFFFF"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">item_type_id
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Consolas"/>
-              <i val="1"/>
-              <color rgb="00D8F3DC"/>
-              <sz val="9"/>
-            </rPr>
-            <t>int32[ref:item_type.id]</t>
-          </r>
+          <t>ItemTypeId
+int32[ref:ItemType.Id]</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <rFont val="Segoe UI"/>
-              <b val="1"/>
-              <color rgb="00FFFFFF"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">drop_range
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Consolas"/>
-              <i val="1"/>
-              <color rgb="00D8F3DC"/>
-              <sz val="9"/>
-            </rPr>
-            <t>DropRange</t>
-          </r>
-        </is>
-      </c>
-      <c r="G1" s="4" t="n"/>
+          <t>DropRange
+Droprange</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="n"/>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <rFont val="Segoe UI"/>
-              <b val="1"/>
-              <color rgb="00FFFFFF"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">tags
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Consolas"/>
-              <i val="1"/>
-              <color rgb="00D8F3DC"/>
-              <sz val="9"/>
-            </rPr>
-            <t>array&lt;int32&gt;</t>
-          </r>
+          <t>Tags
+array&lt;int32&gt;</t>
         </is>
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <rFont val="Segoe UI"/>
-              <b val="1"/>
-              <color rgb="00FFFFFF"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">is_active
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Consolas"/>
-              <i val="1"/>
-              <color rgb="00D8F3DC"/>
-              <sz val="9"/>
-            </rPr>
-            <t>bool</t>
-          </r>
+          <t>IsActive
+bool</t>
         </is>
       </c>
     </row>
     <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="4" t="n"/>
-      <c r="B2" s="4" t="n"/>
-      <c r="C2" s="4" t="n"/>
-      <c r="D2" s="4" t="n"/>
-      <c r="E2" s="4" t="n"/>
+      <c r="A2" s="7" t="n"/>
+      <c r="B2" s="7" t="n"/>
+      <c r="C2" s="7" t="n"/>
+      <c r="D2" s="7" t="n"/>
+      <c r="E2" s="7" t="n"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <rFont val="Segoe UI"/>
-              <b val="1"/>
-              <color rgb="00FFFFFF"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">min
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Consolas"/>
-              <i val="1"/>
-              <color rgb="00D8F3DC"/>
-              <sz val="9"/>
-            </rPr>
-            <t>int32</t>
-          </r>
+          <t>Min
+int32</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <r>
-            <rPr>
-              <rFont val="Segoe UI"/>
-              <b val="1"/>
-              <color rgb="00FFFFFF"/>
-              <sz val="12"/>
-            </rPr>
-            <t xml:space="preserve">max
-</t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Consolas"/>
-              <i val="1"/>
-              <color rgb="00D8F3DC"/>
-              <sz val="9"/>
-            </rPr>
-            <t>int32</t>
-          </r>
-        </is>
-      </c>
-      <c r="H2" s="4" t="n"/>
-      <c r="I2" s="4" t="n"/>
+          <t>Max
+int32</t>
+        </is>
+      </c>
+      <c r="H2" s="7" t="n"/>
+      <c r="I2" s="7" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -781,7 +655,7 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>道具类型，关联 item_type.id</t>
+          <t>道具类型，关联 ItemType.Id</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
@@ -805,16 +679,155 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>药水</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>101,102</t>
+        </is>
+      </c>
+      <c r="I4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>铁剑</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>100</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>201</t>
+        </is>
+      </c>
+      <c r="I5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>魔法石</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>250</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>epic</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>3</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>301,302,303</t>
+        </is>
+      </c>
+      <c r="I6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>面包</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>10</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>101</t>
+        </is>
+      </c>
+      <c r="I7" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="I1:I2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="D1:D2"/>
     <mergeCell ref="E1:E2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="F1:G1"/>
     <mergeCell ref="H1:H2"/>
-    <mergeCell ref="F1:G1"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>
   <conditionalFormatting sqref="A4:I1000">

</xml_diff>